<commit_message>
Noņemti testa dati no excel
</commit_message>
<xml_diff>
--- a/Aptaujas rezultats_Gramzda_IP.xlsx
+++ b/Aptaujas rezultats_Gramzda_IP.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Gramzda_aptauja\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Majas_lapas\Ipadome_Gramzda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC32C814-D43E-435F-8A32-A8CF638785B1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77B9A83-E795-4A1B-BAB6-AF47190070E6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4725" yWindow="2445" windowWidth="21600" windowHeight="11295" xr2:uid="{6E587DD8-68A4-4455-8797-99770335D4CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6E587DD8-68A4-4455-8797-99770335D4CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Dati" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="158">
   <si>
     <t>Respondenta ID</t>
   </si>
@@ -507,9 +507,6 @@
   <si>
     <t>5.2 Kontaktinformācija</t>
   </si>
-  <si>
-    <t>Mājas lapa</t>
-  </si>
 </sst>
 </file>
 
@@ -3751,918 +3748,328 @@
       <c r="BL1" s="2"/>
     </row>
     <row r="2" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="A2" s="20">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4">
-        <v>3</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4">
-        <v>1</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>1</v>
-      </c>
-      <c r="H2" s="4">
-        <v>0</v>
-      </c>
-      <c r="I2" s="4">
-        <v>1</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="K2" s="4">
-        <v>1</v>
-      </c>
-      <c r="L2" s="4">
-        <v>1</v>
-      </c>
-      <c r="M2" s="4">
-        <v>1</v>
-      </c>
-      <c r="N2" s="4">
-        <v>0</v>
-      </c>
-      <c r="O2" s="4">
-        <v>1</v>
-      </c>
-      <c r="P2" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="4">
-        <v>1</v>
-      </c>
-      <c r="R2" s="4">
-        <v>1</v>
-      </c>
-      <c r="S2" s="4">
-        <v>0</v>
-      </c>
-      <c r="T2" s="4">
-        <v>0</v>
-      </c>
-      <c r="U2" s="4">
-        <v>1</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="X2" s="4">
-        <v>4</v>
-      </c>
-      <c r="Y2" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AC2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AD2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AF2" s="4">
-        <v>0</v>
-      </c>
+      <c r="A2" s="20"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
       <c r="AG2" s="4"/>
-      <c r="AH2" s="4">
-        <v>5</v>
-      </c>
-      <c r="AI2" s="4">
-        <v>4</v>
-      </c>
-      <c r="AJ2" s="4">
-        <v>5</v>
-      </c>
-      <c r="AK2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AL2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AM2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AN2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AO2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AQ2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AR2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AS2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AT2" s="4">
-        <v>0</v>
-      </c>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="4"/>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
+      <c r="AL2" s="4"/>
+      <c r="AM2" s="4"/>
+      <c r="AN2" s="4"/>
+      <c r="AO2" s="4"/>
+      <c r="AP2" s="4"/>
+      <c r="AQ2" s="4"/>
+      <c r="AR2" s="4"/>
+      <c r="AS2" s="4"/>
+      <c r="AT2" s="4"/>
       <c r="AU2" s="4"/>
-      <c r="AV2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="AW2" s="4">
-        <v>3</v>
-      </c>
-      <c r="AX2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AY2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AZ2" s="4">
-        <v>1</v>
-      </c>
-      <c r="BA2" s="4">
-        <v>0</v>
-      </c>
-      <c r="BB2" s="4">
-        <v>0</v>
-      </c>
-      <c r="BC2" s="4">
-        <v>1</v>
-      </c>
-      <c r="BD2" s="4">
-        <v>1</v>
-      </c>
-      <c r="BE2" s="4">
-        <v>1</v>
-      </c>
-      <c r="BF2" s="4">
-        <v>0</v>
-      </c>
+      <c r="AV2" s="4"/>
+      <c r="AW2" s="4"/>
+      <c r="AX2" s="4"/>
+      <c r="AY2" s="4"/>
+      <c r="AZ2" s="4"/>
+      <c r="BA2" s="4"/>
+      <c r="BB2" s="4"/>
+      <c r="BC2" s="4"/>
+      <c r="BD2" s="4"/>
+      <c r="BE2" s="4"/>
+      <c r="BF2" s="4"/>
       <c r="BG2" s="4"/>
-      <c r="BH2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="BI2" s="4">
-        <v>3</v>
-      </c>
-      <c r="BJ2" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="BH2" s="4"/>
+      <c r="BI2" s="4"/>
+      <c r="BJ2" s="4"/>
       <c r="BK2" s="21"/>
     </row>
     <row r="3" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="A3" s="20">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4">
-        <v>5</v>
-      </c>
-      <c r="C3" s="4">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4">
-        <v>1</v>
-      </c>
-      <c r="I3" s="4">
-        <v>1</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="K3" s="4">
-        <v>1</v>
-      </c>
-      <c r="L3" s="4">
-        <v>1</v>
-      </c>
-      <c r="M3" s="4">
-        <v>0</v>
-      </c>
-      <c r="N3" s="4">
-        <v>1</v>
-      </c>
-      <c r="O3" s="4">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="4">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4">
-        <v>1</v>
-      </c>
-      <c r="S3" s="4">
-        <v>1</v>
-      </c>
-      <c r="T3" s="4">
-        <v>1</v>
-      </c>
-      <c r="U3" s="4">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="X3" s="4">
-        <v>2</v>
-      </c>
-      <c r="Y3" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AB3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AC3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AE3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="4">
-        <v>0</v>
-      </c>
+      <c r="A3" s="20"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
       <c r="AG3" s="4"/>
-      <c r="AH3" s="4">
-        <v>4</v>
-      </c>
-      <c r="AI3" s="4">
-        <v>3</v>
-      </c>
-      <c r="AJ3" s="4">
-        <v>2</v>
-      </c>
-      <c r="AK3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AL3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AM3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AN3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AO3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AP3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AQ3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AR3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AS3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AT3" s="4">
-        <v>0</v>
-      </c>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+      <c r="AR3" s="4"/>
+      <c r="AS3" s="4"/>
+      <c r="AT3" s="4"/>
       <c r="AU3" s="4"/>
-      <c r="AV3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="AW3" s="4">
-        <v>2</v>
-      </c>
-      <c r="AX3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AY3" s="4">
-        <v>1</v>
-      </c>
-      <c r="AZ3" s="4">
-        <v>1</v>
-      </c>
-      <c r="BA3" s="4">
-        <v>1</v>
-      </c>
-      <c r="BB3" s="4">
-        <v>0</v>
-      </c>
-      <c r="BC3" s="4">
-        <v>0</v>
-      </c>
-      <c r="BD3" s="4">
-        <v>1</v>
-      </c>
-      <c r="BE3" s="4">
-        <v>0</v>
-      </c>
-      <c r="BF3" s="4">
-        <v>1</v>
-      </c>
+      <c r="AV3" s="4"/>
+      <c r="AW3" s="4"/>
+      <c r="AX3" s="4"/>
+      <c r="AY3" s="4"/>
+      <c r="AZ3" s="4"/>
+      <c r="BA3" s="4"/>
+      <c r="BB3" s="4"/>
+      <c r="BC3" s="4"/>
+      <c r="BD3" s="4"/>
+      <c r="BE3" s="4"/>
+      <c r="BF3" s="4"/>
       <c r="BG3" s="4"/>
-      <c r="BH3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="BI3" s="4">
-        <v>2</v>
-      </c>
-      <c r="BJ3" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="BH3" s="4"/>
+      <c r="BI3" s="4"/>
+      <c r="BJ3" s="4"/>
       <c r="BK3" s="21"/>
     </row>
     <row r="4" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4">
-        <v>3</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4">
-        <v>0</v>
-      </c>
-      <c r="M4" s="4">
-        <v>1</v>
-      </c>
-      <c r="N4" s="4">
-        <v>1</v>
-      </c>
-      <c r="O4" s="4">
-        <v>1</v>
-      </c>
-      <c r="P4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4">
-        <v>1</v>
-      </c>
-      <c r="V4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="W4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="X4" s="4">
-        <v>4</v>
-      </c>
-      <c r="Y4" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AA4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AD4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AF4" s="4">
-        <v>0</v>
-      </c>
+      <c r="A4" s="20"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4"/>
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4"/>
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4"/>
+      <c r="AF4" s="4"/>
       <c r="AG4" s="4"/>
-      <c r="AH4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AI4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AJ4" s="4">
-        <v>5</v>
-      </c>
-      <c r="AK4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AL4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AM4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AN4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AO4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AP4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AQ4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AR4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AS4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AT4" s="4">
-        <v>0</v>
-      </c>
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4"/>
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4"/>
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4"/>
+      <c r="AP4" s="4"/>
+      <c r="AQ4" s="4"/>
+      <c r="AR4" s="4"/>
+      <c r="AS4" s="4"/>
+      <c r="AT4" s="4"/>
       <c r="AU4" s="4"/>
-      <c r="AV4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="AW4" s="4">
-        <v>3</v>
-      </c>
-      <c r="AX4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AY4" s="4">
-        <v>1</v>
-      </c>
-      <c r="AZ4" s="4">
-        <v>0</v>
-      </c>
-      <c r="BA4" s="4">
-        <v>0</v>
-      </c>
-      <c r="BB4" s="4">
-        <v>1</v>
-      </c>
-      <c r="BC4" s="4">
-        <v>1</v>
-      </c>
-      <c r="BD4" s="4">
-        <v>0</v>
-      </c>
-      <c r="BE4" s="4">
-        <v>1</v>
-      </c>
-      <c r="BF4" s="4">
-        <v>0</v>
-      </c>
+      <c r="AV4" s="4"/>
+      <c r="AW4" s="4"/>
+      <c r="AX4" s="4"/>
+      <c r="AY4" s="4"/>
+      <c r="AZ4" s="4"/>
+      <c r="BA4" s="4"/>
+      <c r="BB4" s="4"/>
+      <c r="BC4" s="4"/>
+      <c r="BD4" s="4"/>
+      <c r="BE4" s="4"/>
+      <c r="BF4" s="4"/>
       <c r="BG4" s="4"/>
-      <c r="BH4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="BI4" s="4">
-        <v>2</v>
-      </c>
-      <c r="BJ4" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="BH4" s="4"/>
+      <c r="BI4" s="4"/>
+      <c r="BJ4" s="4"/>
       <c r="BK4" s="21"/>
     </row>
     <row r="5" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4">
-        <v>1</v>
-      </c>
-      <c r="I5" s="4">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="K5" s="4">
-        <v>1</v>
-      </c>
-      <c r="L5" s="4">
-        <v>1</v>
-      </c>
-      <c r="M5" s="4">
-        <v>0</v>
-      </c>
-      <c r="N5" s="4">
-        <v>0</v>
-      </c>
-      <c r="O5" s="4">
-        <v>0</v>
-      </c>
-      <c r="P5" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="4">
-        <v>1</v>
-      </c>
-      <c r="R5" s="4">
-        <v>1</v>
-      </c>
-      <c r="S5" s="4">
-        <v>1</v>
-      </c>
-      <c r="T5" s="4">
-        <v>1</v>
-      </c>
-      <c r="U5" s="4">
-        <v>1</v>
-      </c>
-      <c r="V5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="W5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="X5" s="4">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="4">
-        <v>1</v>
-      </c>
+      <c r="A5" s="20"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
+      <c r="AF5" s="4"/>
       <c r="AG5" s="4"/>
-      <c r="AH5" s="4">
-        <v>2</v>
-      </c>
-      <c r="AI5" s="4">
-        <v>2</v>
-      </c>
-      <c r="AJ5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AK5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AL5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AN5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AQ5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AS5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AT5" s="4">
-        <v>1</v>
-      </c>
+      <c r="AH5" s="4"/>
+      <c r="AI5" s="4"/>
+      <c r="AJ5" s="4"/>
+      <c r="AK5" s="4"/>
+      <c r="AL5" s="4"/>
+      <c r="AM5" s="4"/>
+      <c r="AN5" s="4"/>
+      <c r="AO5" s="4"/>
+      <c r="AP5" s="4"/>
+      <c r="AQ5" s="4"/>
+      <c r="AR5" s="4"/>
+      <c r="AS5" s="4"/>
+      <c r="AT5" s="4"/>
       <c r="AU5" s="4"/>
-      <c r="AV5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="AW5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AX5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AY5" s="4">
-        <v>1</v>
-      </c>
-      <c r="AZ5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BA5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BB5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BC5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BD5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BE5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BF5" s="4">
-        <v>1</v>
-      </c>
+      <c r="AV5" s="4"/>
+      <c r="AW5" s="4"/>
+      <c r="AX5" s="4"/>
+      <c r="AY5" s="4"/>
+      <c r="AZ5" s="4"/>
+      <c r="BA5" s="4"/>
+      <c r="BB5" s="4"/>
+      <c r="BC5" s="4"/>
+      <c r="BD5" s="4"/>
+      <c r="BE5" s="4"/>
+      <c r="BF5" s="4"/>
       <c r="BG5" s="4"/>
-      <c r="BH5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="BI5" s="4">
-        <v>1</v>
-      </c>
-      <c r="BJ5" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="BH5" s="4"/>
+      <c r="BI5" s="4"/>
+      <c r="BJ5" s="4"/>
       <c r="BK5" s="21"/>
     </row>
     <row r="6" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4">
-        <v>3</v>
-      </c>
-      <c r="C6" s="4">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>1</v>
-      </c>
-      <c r="H6" s="4">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4">
-        <v>1</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="K6" s="4">
-        <v>1</v>
-      </c>
-      <c r="L6" s="4">
-        <v>1</v>
-      </c>
-      <c r="M6" s="4">
-        <v>1</v>
-      </c>
-      <c r="N6" s="4">
-        <v>0</v>
-      </c>
-      <c r="O6" s="4">
-        <v>1</v>
-      </c>
-      <c r="P6" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4">
-        <v>1</v>
-      </c>
-      <c r="R6" s="4">
-        <v>1</v>
-      </c>
-      <c r="S6" s="4">
-        <v>0</v>
-      </c>
-      <c r="T6" s="4">
-        <v>0</v>
-      </c>
-      <c r="U6" s="4">
-        <v>1</v>
-      </c>
-      <c r="V6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="W6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="X6" s="4">
-        <v>4</v>
-      </c>
-      <c r="Y6" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AA6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AC6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AD6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AF6" s="4">
-        <v>0</v>
-      </c>
+      <c r="A6" s="20"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="4"/>
+      <c r="AB6" s="4"/>
+      <c r="AC6" s="4"/>
+      <c r="AD6" s="4"/>
+      <c r="AE6" s="4"/>
+      <c r="AF6" s="4"/>
       <c r="AG6" s="4"/>
-      <c r="AH6" s="4">
-        <v>5</v>
-      </c>
-      <c r="AI6" s="4">
-        <v>4</v>
-      </c>
-      <c r="AJ6" s="4">
-        <v>5</v>
-      </c>
-      <c r="AK6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AL6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AM6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AN6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AO6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AP6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AQ6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AR6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AS6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AT6" s="4">
-        <v>0</v>
-      </c>
+      <c r="AH6" s="4"/>
+      <c r="AI6" s="4"/>
+      <c r="AJ6" s="4"/>
+      <c r="AK6" s="4"/>
+      <c r="AL6" s="4"/>
+      <c r="AM6" s="4"/>
+      <c r="AN6" s="4"/>
+      <c r="AO6" s="4"/>
+      <c r="AP6" s="4"/>
+      <c r="AQ6" s="4"/>
+      <c r="AR6" s="4"/>
+      <c r="AS6" s="4"/>
+      <c r="AT6" s="4"/>
       <c r="AU6" s="4"/>
-      <c r="AV6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="AW6" s="4">
-        <v>3</v>
-      </c>
-      <c r="AX6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AY6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AZ6" s="4">
-        <v>1</v>
-      </c>
-      <c r="BA6" s="4">
-        <v>0</v>
-      </c>
-      <c r="BB6" s="4">
-        <v>0</v>
-      </c>
-      <c r="BC6" s="4">
-        <v>1</v>
-      </c>
-      <c r="BD6" s="4">
-        <v>1</v>
-      </c>
-      <c r="BE6" s="4">
-        <v>1</v>
-      </c>
-      <c r="BF6" s="4">
-        <v>0</v>
-      </c>
+      <c r="AV6" s="4"/>
+      <c r="AW6" s="4"/>
+      <c r="AX6" s="4"/>
+      <c r="AY6" s="4"/>
+      <c r="AZ6" s="4"/>
+      <c r="BA6" s="4"/>
+      <c r="BB6" s="4"/>
+      <c r="BC6" s="4"/>
+      <c r="BD6" s="4"/>
+      <c r="BE6" s="4"/>
+      <c r="BF6" s="4"/>
       <c r="BG6" s="4"/>
-      <c r="BH6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="BI6" s="4">
-        <v>3</v>
-      </c>
-      <c r="BJ6" s="4" t="s">
-        <v>158</v>
-      </c>
+      <c r="BH6" s="4"/>
+      <c r="BI6" s="4"/>
+      <c r="BJ6" s="4"/>
       <c r="BK6" s="21"/>
     </row>
     <row r="7" spans="1:64" x14ac:dyDescent="0.25">

</xml_diff>